<commit_message>
update critical - coins and problems
</commit_message>
<xml_diff>
--- a/master/pokemonTable_HatchMon_Canonical_v2.xlsx
+++ b/master/pokemonTable_HatchMon_Canonical_v2.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jomipujol/Desktop/PER_JOMI/HATCH.MON/master/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jomipujol/Desktop/PER_JOMI/HATCH.MON/hatch.mon-git/master/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{299AD7BC-FD64-E741-900C-F18301AF8568}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48AC806E-DB78-7D43-B49C-CCAA03C75D8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20" yWindow="660" windowWidth="29400" windowHeight="17020" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="33880" yWindow="1500" windowWidth="29400" windowHeight="17020" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12741" uniqueCount="2930">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12742" uniqueCount="2930">
   <si>
     <t>Hatch.mon canonical Pokémon data</t>
   </si>
@@ -72891,10 +72891,14 @@
       <c r="C2" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="D2" s="2"/>
+      <c r="D2" s="2">
+        <v>1.5</v>
+      </c>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
+      <c r="G2" s="2">
+        <v>40</v>
+      </c>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
@@ -72918,12 +72922,18 @@
       <c r="C3" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="D3" s="2"/>
+      <c r="D3" s="2">
+        <v>3</v>
+      </c>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
+      <c r="G3" s="2">
+        <v>70</v>
+      </c>
       <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
+      <c r="I3" s="2">
+        <v>2</v>
+      </c>
       <c r="J3" s="2"/>
       <c r="K3" s="2"/>
       <c r="L3" s="2"/>
@@ -72945,11 +72955,15 @@
       <c r="C4" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="D4" s="2"/>
+      <c r="D4" s="2">
+        <v>1.5</v>
+      </c>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
+      <c r="H4" s="2">
+        <v>40</v>
+      </c>
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
@@ -72972,12 +72986,18 @@
       <c r="C5" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="D5" s="2"/>
+      <c r="D5" s="2">
+        <v>3</v>
+      </c>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
+      <c r="H5" s="2">
+        <v>70</v>
+      </c>
+      <c r="I5" s="2">
+        <v>2</v>
+      </c>
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
       <c r="L5" s="2"/>
@@ -72999,9 +73019,13 @@
       <c r="C6" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="D6" s="2"/>
+      <c r="D6" s="2">
+        <v>1.5</v>
+      </c>
       <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
+      <c r="F6" s="2">
+        <v>40</v>
+      </c>
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
@@ -73026,12 +73050,18 @@
       <c r="C7" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="D7" s="2"/>
+      <c r="D7" s="2">
+        <v>3</v>
+      </c>
       <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
+      <c r="F7" s="2">
+        <v>70</v>
+      </c>
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
+      <c r="I7" s="2">
+        <v>2</v>
+      </c>
       <c r="J7" s="2"/>
       <c r="K7" s="2"/>
       <c r="L7" s="2"/>
@@ -74053,13 +74083,17 @@
       <c r="C44" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="D44" s="2"/>
+      <c r="D44" s="2">
+        <v>2</v>
+      </c>
       <c r="E44" s="2"/>
       <c r="F44" s="2"/>
       <c r="G44" s="2"/>
       <c r="H44" s="2"/>
       <c r="I44" s="2"/>
-      <c r="J44" s="2"/>
+      <c r="J44" s="2" t="s">
+        <v>2401</v>
+      </c>
       <c r="K44" s="2"/>
       <c r="L44" s="2"/>
       <c r="M44" s="2"/>
@@ -74161,9 +74195,13 @@
       <c r="C48" s="2" t="s">
         <v>232</v>
       </c>
-      <c r="D48" s="2"/>
+      <c r="D48" s="2">
+        <v>1</v>
+      </c>
       <c r="E48" s="2"/>
-      <c r="F48" s="2"/>
+      <c r="F48" s="2">
+        <v>50</v>
+      </c>
       <c r="G48" s="2"/>
       <c r="H48" s="2"/>
       <c r="I48" s="2"/>
@@ -74188,12 +74226,18 @@
       <c r="C49" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="D49" s="2"/>
+      <c r="D49" s="2">
+        <v>2.5</v>
+      </c>
       <c r="E49" s="2"/>
-      <c r="F49" s="2"/>
+      <c r="F49" s="2">
+        <v>80</v>
+      </c>
       <c r="G49" s="2"/>
       <c r="H49" s="2"/>
-      <c r="I49" s="2"/>
+      <c r="I49" s="2">
+        <v>2</v>
+      </c>
       <c r="J49" s="2"/>
       <c r="K49" s="2"/>
       <c r="L49" s="2"/>
@@ -75635,8 +75679,12 @@
       <c r="C100" s="2" t="s">
         <v>459</v>
       </c>
-      <c r="D100" s="2"/>
-      <c r="E100" s="2"/>
+      <c r="D100" s="2">
+        <v>2</v>
+      </c>
+      <c r="E100" s="2">
+        <v>70</v>
+      </c>
       <c r="F100" s="2"/>
       <c r="G100" s="2"/>
       <c r="H100" s="2"/>
@@ -75662,12 +75710,16 @@
       <c r="C101" s="2" t="s">
         <v>461</v>
       </c>
-      <c r="D101" s="2"/>
+      <c r="D101" s="2">
+        <v>3.5</v>
+      </c>
       <c r="E101" s="2"/>
       <c r="F101" s="2"/>
       <c r="G101" s="2"/>
       <c r="H101" s="2"/>
-      <c r="I101" s="2"/>
+      <c r="I101" s="2">
+        <v>5</v>
+      </c>
       <c r="J101" s="2"/>
       <c r="K101" s="2"/>
       <c r="L101" s="2"/>

</xml_diff>